<commit_message>
Rename agent: Cheshire Cat -> Reconciliation Agent (customer/RM names preserved)
</commit_message>
<xml_diff>
--- a/cheshire_reconciliation_2026-04-22.xlsx
+++ b/cheshire_reconciliation_2026-04-22.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://m365x97078969-my.sharepoint.com/personal/sysadmin_wondercorp_jp/Documents/2. Management/Reconciliation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EF237BB1-CAED-4053-A8B5-517F69F7B039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F97E9AD-31DF-4AFD-A47F-414D0C448A5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15450" activeTab="3" xr2:uid="{253D5BF4-788E-489A-A550-95F3355295FC}"/>
+    <workbookView xWindow="7030" yWindow="4710" windowWidth="28800" windowHeight="15450" activeTab="3" xr2:uid="{BF73B4A3-184C-4AAD-BFFD-1BFFD05312CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Mainframe TRANLIST" sheetId="1" r:id="rId1"/>
@@ -422,7 +422,7 @@
     <t>RECONCILIATION RESULT - 2026-04-22</t>
   </si>
   <si>
-    <t>Generated by Cheshire Cat at 08:04:17 UTC  |  3 mismatches found across 15 mainframe transactions / 8 portal settlements / 10 D365 customers.</t>
+    <t>Generated by Reconciliation Agent at 08:04:17 UTC  |  3 mismatches found across 15 mainframe transactions / 8 portal settlements / 10 D365 customers.</t>
   </si>
   <si>
     <t>#</t>
@@ -989,7 +989,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAA50528-2A66-4A13-A27B-DB9344F9F7D5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62D9D35E-DDB4-4868-A716-01E36D302560}">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1412,7 +1412,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B692F1FE-4FB5-4781-9BC8-BF82D078C299}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436B5592-B4EA-466C-9283-BEC2A31BA0D4}">
   <dimension ref="A1:D22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1638,7 +1638,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{377CC456-68ED-4B69-80D8-E0B716F77AD6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D4DF733-45AD-495B-AAC1-DDD828F73DEC}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1942,7 +1942,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CEBB082D-B6E5-4AD8-8EF0-723ED29DF363}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05A2A782-A32E-40F6-9077-58483554D490}">
   <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>